<commit_message>
Actualiza planillas del Sprint 2 y Product Backlog
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjzVJTSwK1GxUk7siw2Qgf
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Sprint 2/Burndown-S2.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Sprint 2/Burndown-S2.xlsx
@@ -16,11 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0;[RED]\-0.0;0"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -837,7 +836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:GR200"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="17" min="1" max="1"/>
@@ -867,7 +866,7 @@
         </is>
       </c>
       <c r="C3" s="22" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" s="18"/>
@@ -903,7 +902,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="18">
+    <row r="6" ht="58" customHeight="1" s="18">
       <c r="A6" s="24" t="n">
         <v>1</v>
       </c>
@@ -915,7 +914,7 @@
         <v/>
       </c>
       <c r="D6" s="26" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E6" s="27">
         <f>IF(D6="","",D6-C6)</f>
@@ -923,7 +922,7 @@
       </c>
       <c r="F6" s="28" t="inlineStr">
         <is>
-          <t>Corte 5 oct según Trello: PC-PRO-01 y PC-PRO-02 en Hecho (7 pts). Recalculado con 65 pts (eran 50 de 57).</t>
+          <t>Corte 5 oct según Trello: PC-PRO-01 y PC-PRO-02 en Hecho (7 pts). Recalculado con 70 pts (eran 50 de 57; luego 58 de 65).</t>
         </is>
       </c>
     </row>
@@ -939,7 +938,7 @@
         <v/>
       </c>
       <c r="D7" s="26" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E7" s="27">
         <f>IF(D7="","",D7-C7)</f>
@@ -963,7 +962,7 @@
         <v/>
       </c>
       <c r="D8" s="26" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E8" s="27">
         <f>IF(D8="","",D8-C8)</f>
@@ -987,7 +986,7 @@
         <v/>
       </c>
       <c r="D9" s="26" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E9" s="27">
         <f>IF(D9="","",D9-C9)</f>
@@ -1011,7 +1010,7 @@
         <v/>
       </c>
       <c r="D10" s="26" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E10" s="27">
         <f>IF(D10="","",D10-C10)</f>
@@ -1023,7 +1022,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" s="18">
+    <row r="11" ht="58" customHeight="1" s="18">
       <c r="A11" s="24" t="n">
         <v>6</v>
       </c>
@@ -1035,7 +1034,7 @@
         <v/>
       </c>
       <c r="D11" s="26" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E11" s="27">
         <f>IF(D11="","",D11-C11)</f>
@@ -1043,7 +1042,7 @@
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
-          <t>13 oct: PC-IA-01 (8 pts) se incorpora al sprint; sigue sin validar. Quedan 58 pts.</t>
+          <t>13 oct: PC-IA-01 (8 pts) se incorpora al sprint. Recalculado con PC-AUT-07 (70 pts): quedan 63.</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1057,9 @@
         <f>ROUND($C$3-$C$3*(A12-1)/(14-1),1)</f>
         <v/>
       </c>
-      <c r="D12" s="26" t="n"/>
+      <c r="D12" s="26" t="n">
+        <v>63</v>
+      </c>
       <c r="E12" s="27">
         <f>IF(D12="","",D12-C12)</f>
         <v/>
@@ -1076,7 +1077,9 @@
         <f>ROUND($C$3-$C$3*(A13-1)/(14-1),1)</f>
         <v/>
       </c>
-      <c r="D13" s="26" t="n"/>
+      <c r="D13" s="26" t="n">
+        <v>63</v>
+      </c>
       <c r="E13" s="27">
         <f>IF(D13="","",D13-C13)</f>
         <v/>
@@ -1094,7 +1097,9 @@
         <f>ROUND($C$3-$C$3*(A14-1)/(14-1),1)</f>
         <v/>
       </c>
-      <c r="D14" s="26" t="n"/>
+      <c r="D14" s="26" t="n">
+        <v>63</v>
+      </c>
       <c r="E14" s="27">
         <f>IF(D14="","",D14-C14)</f>
         <v/>
@@ -1112,14 +1117,16 @@
         <f>ROUND($C$3-$C$3*(A15-1)/(14-1),1)</f>
         <v/>
       </c>
-      <c r="D15" s="26" t="n"/>
+      <c r="D15" s="26" t="n">
+        <v>63</v>
+      </c>
       <c r="E15" s="27">
         <f>IF(D15="","",D15-C15)</f>
         <v/>
       </c>
       <c r="F15" s="28" t="n"/>
     </row>
-    <row r="16" ht="15" customHeight="1" s="18">
+    <row r="16" ht="58" customHeight="1" s="18">
       <c r="A16" s="24" t="n">
         <v>11</v>
       </c>
@@ -1130,12 +1137,18 @@
         <f>ROUND($C$3-$C$3*(A16-1)/(14-1),1)</f>
         <v/>
       </c>
-      <c r="D16" s="26" t="n"/>
+      <c r="D16" s="26" t="n">
+        <v>5</v>
+      </c>
       <c r="E16" s="27">
         <f>IF(D16="","",D16-C16)</f>
         <v/>
       </c>
-      <c r="F16" s="28" t="n"/>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>Reunión interna (Felipe, Esteban y Christian): se dan por Hecho PC-AUT-04, PC-AUT-05, PC-TEC-04, PC-COT-01, PC-COT-02, PC-CLI-01 y PC-CLI-02 (50 pts) y PC-IA-01 (8 pts). Quedan 5 pts (PC-AUT-07).</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="18">
       <c r="A17" s="24" t="n">
@@ -1148,14 +1161,20 @@
         <f>ROUND($C$3-$C$3*(A17-1)/(14-1),1)</f>
         <v/>
       </c>
-      <c r="D17" s="26" t="n"/>
+      <c r="D17" s="26" t="n">
+        <v>5</v>
+      </c>
       <c r="E17" s="27">
         <f>IF(D17="","",D17-C17)</f>
         <v/>
       </c>
-      <c r="F17" s="28" t="n"/>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="18">
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>Sin historias nuevas en Hecho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1" s="18">
       <c r="A18" s="24" t="n">
         <v>13</v>
       </c>
@@ -1166,12 +1185,18 @@
         <f>ROUND($C$3-$C$3*(A18-1)/(14-1),1)</f>
         <v/>
       </c>
-      <c r="D18" s="26" t="n"/>
+      <c r="D18" s="26" t="n">
+        <v>5</v>
+      </c>
       <c r="E18" s="27">
         <f>IF(D18="","",D18-C18)</f>
         <v/>
       </c>
-      <c r="F18" s="28" t="n"/>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>22 oct: PC-AUT-07 (5 pts) se incorpora al sprint (65 → 70) y queda En proceso. Las tarjetas se movieron en Trello hoy; el burndown usa la fecha de la decisión (20 oct).</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="18">
       <c r="A19" s="24" t="n">
@@ -1305,10 +1330,10 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="25.5" customHeight="1" s="18">
+    <row r="33" ht="58" customHeight="1" s="18">
       <c r="A33" s="36" t="inlineStr">
         <is>
-          <t>• Comprometidos: 65 pts = 57 pts originales + PC-IA-01 (8 pts), adelantada del Sprint 4 el 13 oct por decisión del equipo. Los días 1 a 5 se recalcularon con el nuevo total (58 pts restantes, antes 50 de 57) para que el ideal y el real sean comparables. PC-TEC-03 sigue fuera del alcance.</t>
+          <t>• Comprometidos: 70 pts = 57 pts originales + PC-IA-01 (8 pts), adelantada del Sprint 4 el 13 oct por decisión del equipo, + PC-AUT-07 (5 pts), incorporada el 22 oct. Los días 1 a 10 se recalcularon con el nuevo total (63 pts restantes) para que el ideal y el real sean comparables. PC-TEC-03 sigue fuera del alcance.</t>
         </is>
       </c>
     </row>
@@ -1319,10 +1344,10 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="25.5" customHeight="1" s="18">
+    <row r="35" ht="72" customHeight="1" s="18">
       <c r="A35" s="36" t="inlineStr">
         <is>
-          <t>• Los puntos se queman solo cuando la tarjeta está en Hecho en Trello. Historias con avance construido pero aún sin validar (COT-01/02, CLI-02, AUT-05, TEC-04) o en revisión (CLI-01, AUT-04) no restan puntos todavía. PC-IA-01 (construida, sin validar; casos CP-057, CP-061 y CP-062 por ejecutar) tampoco resta.</t>
+          <t>• Los puntos se queman cuando la historia está en Hecho. Las tarjetas En revisión se dieron por hechas en la reunión del martes 20 oct (Felipe, Esteban y Christian) y se movieron en Trello el 22 oct; se registra el 20 oct. PC-IA-01 se da por hecha (técnicamente lista) pese al problema de cobros de la API de Gemini (Impediment Log I-007); sus casos CP-057, CP-061 y CP-062 no tienen ejecución registrada. PC-AUT-07 (5 pts) sigue en proceso.</t>
         </is>
       </c>
     </row>
@@ -1351,24 +1376,23 @@
     <row r="58" s="18"/>
     <row r="59" s="18"/>
     <row r="60" s="18"/>
-    <row r="200"/>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A22:B22"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:E19">
     <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1">

</xml_diff>